<commit_message>
added tests with their status
</commit_message>
<xml_diff>
--- a/testData.xlsx
+++ b/testData.xlsx
@@ -3,19 +3,22 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30326"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0DE48A5-40E6-46B2-B72F-0C212F444E3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FDB3DC2D-73EB-444D-BBE4-5CB249694284}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$E$1:$E$31</definedName>
+  </definedNames>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="156" uniqueCount="59">
   <si>
     <t>start location</t>
   </si>
@@ -111,13 +114,97 @@
   </si>
   <si>
     <t>15:07:00</t>
+  </si>
+  <si>
+    <t>ehvbst</t>
+  </si>
+  <si>
+    <t>05:03:00</t>
+  </si>
+  <si>
+    <t>05:07:00</t>
+  </si>
+  <si>
+    <t>material trip</t>
+  </si>
+  <si>
+    <t>ehvapt</t>
+  </si>
+  <si>
+    <t>05:31:00</t>
+  </si>
+  <si>
+    <t>service trip</t>
+  </si>
+  <si>
+    <t>06:04:00</t>
+  </si>
+  <si>
+    <t>idle</t>
+  </si>
+  <si>
+    <t>06:29:00</t>
+  </si>
+  <si>
+    <t>06:31:00</t>
+  </si>
+  <si>
+    <t>06:55:00</t>
+  </si>
+  <si>
+    <t>06:56:00</t>
+  </si>
+  <si>
+    <t>07:21:00</t>
+  </si>
+  <si>
+    <t>07:45:00</t>
+  </si>
+  <si>
+    <t>07:46:00</t>
+  </si>
+  <si>
+    <t>08:11:00</t>
+  </si>
+  <si>
+    <t>08:31:00</t>
+  </si>
+  <si>
+    <t>08:36:00</t>
+  </si>
+  <si>
+    <t>09:01:00</t>
+  </si>
+  <si>
+    <t>09:21:00</t>
+  </si>
+  <si>
+    <t>09:26:00</t>
+  </si>
+  <si>
+    <t>09:51:00</t>
+  </si>
+  <si>
+    <t>10:11:00</t>
+  </si>
+  <si>
+    <t>10:16:00</t>
+  </si>
+  <si>
+    <t>10:41:00</t>
+  </si>
+  <si>
+    <t>11:01:00</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <numFmts count="1">
+    <numFmt numFmtId="165" formatCode="[$-F400]h:mm:ss\ am/pm"/>
+  </numFmts>
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -130,6 +217,13 @@
       <sz val="11"/>
       <name val="Calibri"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -167,11 +261,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="21" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -511,7 +608,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H12"/>
+  <dimension ref="A1:H31"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="24" width="13.54296875" customWidth="1"/>
@@ -727,26 +824,26 @@
         <v>4</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A10" t="s">
-        <v>8</v>
-      </c>
-      <c r="B10" t="s">
-        <v>8</v>
-      </c>
-      <c r="C10" t="s">
+    <row r="10" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A10" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C10" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="D10" t="s">
+      <c r="D10" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="E10" t="s">
+      <c r="E10" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="G10">
-        <v>-150</v>
-      </c>
-      <c r="H10">
+      <c r="G10" s="2">
+        <v>150</v>
+      </c>
+      <c r="H10" s="2">
         <v>5</v>
       </c>
     </row>
@@ -767,7 +864,7 @@
         <v>11</v>
       </c>
       <c r="G11">
-        <v>-180</v>
+        <v>0</v>
       </c>
       <c r="H11">
         <v>6</v>
@@ -796,7 +893,472 @@
         <v>7</v>
       </c>
     </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
+        <v>8</v>
+      </c>
+      <c r="B13" t="s">
+        <v>32</v>
+      </c>
+      <c r="C13" t="s">
+        <v>33</v>
+      </c>
+      <c r="D13" t="s">
+        <v>34</v>
+      </c>
+      <c r="E13" t="s">
+        <v>35</v>
+      </c>
+      <c r="G13">
+        <v>1.98</v>
+      </c>
+      <c r="H13">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A14" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="F14" s="2">
+        <v>401</v>
+      </c>
+      <c r="G14" s="2">
+        <v>-10.803599999999999</v>
+      </c>
+      <c r="H14" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A15" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="E15" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="G15" s="2">
+        <v>-5</v>
+      </c>
+      <c r="H15" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A16" t="s">
+        <v>36</v>
+      </c>
+      <c r="B16" t="s">
+        <v>32</v>
+      </c>
+      <c r="C16" t="s">
+        <v>39</v>
+      </c>
+      <c r="D16" t="s">
+        <v>41</v>
+      </c>
+      <c r="E16" t="s">
+        <v>38</v>
+      </c>
+      <c r="F16">
+        <v>401</v>
+      </c>
+      <c r="G16">
+        <v>10.86</v>
+      </c>
+      <c r="H16">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A17" t="s">
+        <v>32</v>
+      </c>
+      <c r="B17" t="s">
+        <v>32</v>
+      </c>
+      <c r="C17" t="s">
+        <v>41</v>
+      </c>
+      <c r="D17" t="s">
+        <v>42</v>
+      </c>
+      <c r="E17" t="s">
+        <v>40</v>
+      </c>
+      <c r="G17">
+        <v>5</v>
+      </c>
+      <c r="H17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A18" t="s">
+        <v>32</v>
+      </c>
+      <c r="B18" t="s">
+        <v>36</v>
+      </c>
+      <c r="C18" t="s">
+        <v>42</v>
+      </c>
+      <c r="D18" t="s">
+        <v>43</v>
+      </c>
+      <c r="E18" t="s">
+        <v>38</v>
+      </c>
+      <c r="F18">
+        <v>401</v>
+      </c>
+      <c r="G18">
+        <v>10.803599999999999</v>
+      </c>
+      <c r="H18">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A19" t="s">
+        <v>36</v>
+      </c>
+      <c r="B19" t="s">
+        <v>36</v>
+      </c>
+      <c r="C19" t="s">
+        <v>43</v>
+      </c>
+      <c r="D19" t="s">
+        <v>44</v>
+      </c>
+      <c r="E19" t="s">
+        <v>40</v>
+      </c>
+      <c r="G19">
+        <v>5</v>
+      </c>
+      <c r="H19">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A20" t="s">
+        <v>36</v>
+      </c>
+      <c r="B20" t="s">
+        <v>32</v>
+      </c>
+      <c r="C20" t="s">
+        <v>44</v>
+      </c>
+      <c r="D20" t="s">
+        <v>45</v>
+      </c>
+      <c r="E20" t="s">
+        <v>38</v>
+      </c>
+      <c r="F20">
+        <v>401</v>
+      </c>
+      <c r="G20">
+        <v>10.86</v>
+      </c>
+      <c r="H20">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A21" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="D21" s="3">
+        <v>0.30694444444444446</v>
+      </c>
+      <c r="E21" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="G21" s="2">
+        <v>5</v>
+      </c>
+      <c r="H21" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A22" t="s">
+        <v>32</v>
+      </c>
+      <c r="B22" t="s">
+        <v>36</v>
+      </c>
+      <c r="C22" t="s">
+        <v>45</v>
+      </c>
+      <c r="D22" t="s">
+        <v>46</v>
+      </c>
+      <c r="E22" t="s">
+        <v>38</v>
+      </c>
+      <c r="F22">
+        <v>400</v>
+      </c>
+      <c r="G22">
+        <v>12.849600000000001</v>
+      </c>
+      <c r="H22">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A23" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="C23" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="D23" s="4">
+        <v>0.32361111111111113</v>
+      </c>
+      <c r="E23" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="G23" s="2">
+        <v>5</v>
+      </c>
+      <c r="H23" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A24" t="s">
+        <v>36</v>
+      </c>
+      <c r="B24" t="s">
+        <v>32</v>
+      </c>
+      <c r="C24" t="s">
+        <v>47</v>
+      </c>
+      <c r="D24" t="s">
+        <v>48</v>
+      </c>
+      <c r="E24" t="s">
+        <v>38</v>
+      </c>
+      <c r="F24">
+        <v>401</v>
+      </c>
+      <c r="G24">
+        <v>10.86</v>
+      </c>
+      <c r="H24">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A25" t="s">
+        <v>32</v>
+      </c>
+      <c r="B25" t="s">
+        <v>36</v>
+      </c>
+      <c r="C25" t="s">
+        <v>48</v>
+      </c>
+      <c r="D25" t="s">
+        <v>49</v>
+      </c>
+      <c r="E25" t="s">
+        <v>35</v>
+      </c>
+      <c r="G25">
+        <v>10.32</v>
+      </c>
+      <c r="H25">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A26" t="s">
+        <v>36</v>
+      </c>
+      <c r="B26" t="s">
+        <v>32</v>
+      </c>
+      <c r="C26" t="s">
+        <v>50</v>
+      </c>
+      <c r="D26" t="s">
+        <v>51</v>
+      </c>
+      <c r="E26" t="s">
+        <v>38</v>
+      </c>
+      <c r="F26">
+        <v>401</v>
+      </c>
+      <c r="G26">
+        <v>10.86</v>
+      </c>
+      <c r="H26">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A27" t="s">
+        <v>32</v>
+      </c>
+      <c r="B27" t="s">
+        <v>36</v>
+      </c>
+      <c r="C27" t="s">
+        <v>51</v>
+      </c>
+      <c r="D27" t="s">
+        <v>52</v>
+      </c>
+      <c r="E27" t="s">
+        <v>35</v>
+      </c>
+      <c r="G27">
+        <v>10.32</v>
+      </c>
+      <c r="H27">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A28" t="s">
+        <v>36</v>
+      </c>
+      <c r="B28" t="s">
+        <v>32</v>
+      </c>
+      <c r="C28" t="s">
+        <v>53</v>
+      </c>
+      <c r="D28" t="s">
+        <v>54</v>
+      </c>
+      <c r="E28" t="s">
+        <v>38</v>
+      </c>
+      <c r="F28">
+        <v>401</v>
+      </c>
+      <c r="G28">
+        <v>10.86</v>
+      </c>
+      <c r="H28">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A29" t="s">
+        <v>32</v>
+      </c>
+      <c r="B29" t="s">
+        <v>36</v>
+      </c>
+      <c r="C29" t="s">
+        <v>54</v>
+      </c>
+      <c r="D29" t="s">
+        <v>55</v>
+      </c>
+      <c r="E29" t="s">
+        <v>35</v>
+      </c>
+      <c r="G29">
+        <v>10.32</v>
+      </c>
+      <c r="H29">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A30" t="s">
+        <v>36</v>
+      </c>
+      <c r="B30" t="s">
+        <v>32</v>
+      </c>
+      <c r="C30" t="s">
+        <v>56</v>
+      </c>
+      <c r="D30" t="s">
+        <v>57</v>
+      </c>
+      <c r="E30" t="s">
+        <v>38</v>
+      </c>
+      <c r="F30">
+        <v>401</v>
+      </c>
+      <c r="G30">
+        <v>10.86</v>
+      </c>
+      <c r="H30">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A31" t="s">
+        <v>32</v>
+      </c>
+      <c r="B31" t="s">
+        <v>36</v>
+      </c>
+      <c r="C31" t="s">
+        <v>57</v>
+      </c>
+      <c r="D31" t="s">
+        <v>58</v>
+      </c>
+      <c r="E31" t="s">
+        <v>35</v>
+      </c>
+      <c r="G31">
+        <v>10.32</v>
+      </c>
+      <c r="H31">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
+  <autoFilter ref="E1:E31" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>

</xml_diff>